<commit_message>
Implement initial summary financing dashboard
- Add basic design viewer for existing PNG charts

- Create JSON expansion structure for multiple fuels/models

- Set up foundation for scalable chart generation

- Separate design preview from calculation logic

- Prepare for Excel integration and formula processing
</commit_message>
<xml_diff>
--- a/backend/Rwanda/carbon-credits-general.xlsx
+++ b/backend/Rwanda/carbon-credits-general.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="59.54296875" customWidth="1" min="1" max="1"/>
@@ -651,7 +651,7 @@
     <row r="4" ht="15.5" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CO2 emited - CleanStep scenario</t>
+          <t>CO2 emited - Aligned scenario</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -660,47 +660,47 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>21.61054123063169</v>
+        <v>0</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>19.40524688334832</v>
+        <v>0</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>17.42849567827935</v>
+        <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>15.45174447321038</v>
+        <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>13.47499326814141</v>
+        <v>0</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>11.49824206307243</v>
+        <v>0</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>9.521490858003462</v>
+        <v>0</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>9.104909776724984</v>
+        <v>0</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>9.190097029539562</v>
+        <v>0</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>9.275284282354139</v>
+        <v>0</v>
       </c>
       <c r="M4" s="11" t="n">
-        <v>9.360471535168717</v>
+        <v>0</v>
       </c>
       <c r="N4" s="11" t="n">
-        <v>9.445658787983295</v>
+        <v>0</v>
       </c>
       <c r="O4" s="8" t="n"/>
     </row>
     <row r="5" ht="15.5" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>△▲{model} vs. BAU</t>
+          <t>CO2 emited - CleanStep scenario</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -709,47 +709,47 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0</v>
+        <v>21.61054123063169</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>0</v>
+        <v>19.40524688334832</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>0</v>
+        <v>17.42849567827935</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0</v>
+        <v>15.45174447321038</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>0</v>
+        <v>13.47499326814141</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>0</v>
+        <v>11.49824206307243</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>0</v>
+        <v>9.521490858003462</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>0</v>
+        <v>9.104909776724984</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>0</v>
+        <v>9.190097029539562</v>
       </c>
       <c r="L5" s="11" t="n">
-        <v>0</v>
+        <v>9.275284282354139</v>
       </c>
       <c r="M5" s="11" t="n">
-        <v>0</v>
+        <v>9.360471535168717</v>
       </c>
       <c r="N5" s="11" t="n">
-        <v>0</v>
+        <v>9.445658787983295</v>
       </c>
       <c r="O5" s="8" t="n"/>
     </row>
     <row r="6" ht="15.5" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>△▲CleanStep vs. BAU</t>
+          <t>△▲{model} vs. BAU</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -758,47 +758,47 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-0.0003676442443278916</v>
+        <v>0</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>1.19664580875806</v>
+        <v>0</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>2.409680987577868</v>
+        <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3.622716166397689</v>
+        <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>4.835751345217499</v>
+        <v>0</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>6.04878652403732</v>
+        <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>7.261821702857139</v>
+        <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>7.330782355213785</v>
+        <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>7.176585865682938</v>
+        <v>0</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>7.022389376152081</v>
+        <v>0</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>6.868192886621223</v>
+        <v>0</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>6.713996397090376</v>
+        <v>0</v>
       </c>
       <c r="O6" s="8" t="n"/>
     </row>
     <row r="7" ht="15.5" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>CO2 equivalent avoided in the {model}</t>
+          <t>△▲Aligned vs. BAU</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -847,7 +847,7 @@
     <row r="8" ht="15.5" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CO2 equivalent avoided in the CleanStep</t>
+          <t>△▲CleanStep vs. BAU</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -856,52 +856,52 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0</v>
+        <v>-0.0003676442443278916</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0.957316647006448</v>
+        <v>1.19664580875806</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>1.927744790062295</v>
+        <v>2.409680987577868</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>2.898172933118151</v>
+        <v>3.622716166397689</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>3.868601076174</v>
+        <v>4.835751345217499</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>4.839029219229856</v>
+        <v>6.04878652403732</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>5.809457362285712</v>
+        <v>7.261821702857139</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>5.864625884171028</v>
+        <v>7.330782355213785</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>5.741268692546351</v>
+        <v>7.176585865682938</v>
       </c>
       <c r="L8" s="11" t="n">
-        <v>5.617911500921664</v>
+        <v>7.022389376152081</v>
       </c>
       <c r="M8" s="11" t="n">
-        <v>5.494554309296978</v>
+        <v>6.868192886621223</v>
       </c>
       <c r="N8" s="11" t="n">
-        <v>5.371197117672301</v>
+        <v>6.713996397090376</v>
       </c>
       <c r="O8" s="8" t="n"/>
     </row>
     <row r="9" ht="15.5" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Potential income from Carbon Credits in the {model} Plan - right</t>
+          <t>CO2 equivalent avoided in the {model}</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>M USD</t>
+          <t>CO2Eq MT/y</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
@@ -945,81 +945,277 @@
     <row r="10" ht="15.5" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>CO2 equivalent avoided in the Aligned</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>CO2Eq MT/y</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="15.5" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CO2 equivalent avoided in the CleanStep</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CO2Eq MT/y</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0.957316647006448</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>1.927744790062295</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>2.898172933118151</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>3.868601076174</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>4.839029219229856</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>5.809457362285712</v>
+      </c>
+      <c r="J11" s="11" t="n">
+        <v>5.864625884171028</v>
+      </c>
+      <c r="K11" s="11" t="n">
+        <v>5.741268692546351</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>5.617911500921664</v>
+      </c>
+      <c r="M11" s="11" t="n">
+        <v>5.494554309296978</v>
+      </c>
+      <c r="N11" s="11" t="n">
+        <v>5.371197117672301</v>
+      </c>
+      <c r="O11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="15.5" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Potential income from Carbon Credits in the {model} Plan - right</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>M USD</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Potential income from Carbon Credits in the Aligned Plan - right</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>M USD</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Potential income from Carbon Credits in the CleanStep Plan - right</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>M USD</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="11" t="n">
+      <c r="C14" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="11" t="n">
         <v>9.57316647006448</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E14" s="11" t="n">
         <v>19.27744790062295</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F14" s="11" t="n">
         <v>28.98172933118151</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G14" s="11" t="n">
         <v>38.68601076173999</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H14" s="11" t="n">
         <v>48.39029219229856</v>
       </c>
-      <c r="I10" s="11" t="n">
+      <c r="I14" s="11" t="n">
         <v>58.09457362285712</v>
       </c>
-      <c r="J10" s="11" t="n">
+      <c r="J14" s="11" t="n">
         <v>58.64625884171028</v>
       </c>
-      <c r="K10" s="11" t="n">
+      <c r="K14" s="11" t="n">
         <v>57.4126869254635</v>
       </c>
-      <c r="L10" s="11" t="n">
+      <c r="L14" s="11" t="n">
         <v>56.17911500921664</v>
       </c>
-      <c r="M10" s="11" t="n">
+      <c r="M14" s="11" t="n">
         <v>54.94554309296979</v>
       </c>
-      <c r="N10" s="11" t="n">
+      <c r="N14" s="11" t="n">
         <v>53.71197117672301</v>
       </c>
-      <c r="O10" s="8" t="n"/>
-    </row>
-    <row r="11" ht="15.5" customHeight="1">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
-      <c r="J11" s="10" t="n"/>
-      <c r="K11" s="10" t="n"/>
-      <c r="L11" s="10" t="n"/>
-      <c r="M11" s="10" t="n"/>
-      <c r="N11" s="10" t="n"/>
-      <c r="O11" s="8" t="n"/>
-    </row>
-    <row r="12" ht="15.5" customHeight="1">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
+      <c r="O14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
+      <c r="H15" s="10" t="n"/>
+      <c r="I15" s="10" t="n"/>
+      <c r="J15" s="10" t="n"/>
+      <c r="K15" s="10" t="n"/>
+      <c r="L15" s="10" t="n"/>
+      <c r="M15" s="10" t="n"/>
+      <c r="N15" s="10" t="n"/>
+      <c r="O15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>